<commit_message>
primi script analisi risorsa dominante
</commit_message>
<xml_diff>
--- a/exploratory_data_analysis/dimensions_reduction/risultati/correlazioni_dispersioni/matrice_correlazione.xlsx
+++ b/exploratory_data_analysis/dimensions_reduction/risultati/correlazioni_dispersioni/matrice_correlazione.xlsx
@@ -496,7 +496,7 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>gdp-pop-urban_merged</t>
+          <t>gdp_pop_urban_merged</t>
         </is>
       </c>
     </row>
@@ -546,7 +546,7 @@
         <v>-0.06365188075385719</v>
       </c>
       <c r="O2" t="n">
-        <v>0.4392329713618455</v>
+        <v>0.4392329713618456</v>
       </c>
     </row>
     <row r="3">
@@ -693,7 +693,7 @@
         <v>0.1321416088647652</v>
       </c>
       <c r="O5" t="n">
-        <v>-0.03071466180415533</v>
+        <v>-0.03071466180415534</v>
       </c>
     </row>
     <row r="6">
@@ -742,7 +742,7 @@
         <v>-0.08563968501436756</v>
       </c>
       <c r="O6" t="n">
-        <v>-0.04134193923629654</v>
+        <v>-0.04134193923629658</v>
       </c>
     </row>
     <row r="7">
@@ -840,7 +840,7 @@
         <v>0.03307085724047992</v>
       </c>
       <c r="O8" t="n">
-        <v>0.05515280701772647</v>
+        <v>0.05515280701772651</v>
       </c>
     </row>
     <row r="9">
@@ -987,7 +987,7 @@
         <v>0.01960986702368907</v>
       </c>
       <c r="O11" t="n">
-        <v>-0.008924192964144765</v>
+        <v>-0.008924192964144761</v>
       </c>
     </row>
     <row r="12">
@@ -1036,7 +1036,7 @@
         <v>0.1265143597509155</v>
       </c>
       <c r="O12" t="n">
-        <v>0.01590378690918018</v>
+        <v>0.01590378690918017</v>
       </c>
     </row>
     <row r="13">
@@ -1134,17 +1134,17 @@
         <v>1</v>
       </c>
       <c r="O14" t="n">
-        <v>-0.03422786351058908</v>
+        <v>-0.03422786351058907</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>gdp-pop-urban_merged</t>
+          <t>gdp_pop_urban_merged</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.4392329713618455</v>
+        <v>0.4392329713618456</v>
       </c>
       <c r="C15" t="n">
         <v>0.1940996913778291</v>
@@ -1153,16 +1153,16 @@
         <v>0.0604906980583572</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.03071466180415533</v>
+        <v>-0.03071466180415534</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.04134193923629654</v>
+        <v>-0.04134193923629658</v>
       </c>
       <c r="G15" t="n">
         <v>0.1959009620477364</v>
       </c>
       <c r="H15" t="n">
-        <v>0.05515280701772647</v>
+        <v>0.05515280701772651</v>
       </c>
       <c r="I15" t="n">
         <v>0.02901894782023856</v>
@@ -1171,16 +1171,16 @@
         <v>0.2806493460516831</v>
       </c>
       <c r="K15" t="n">
-        <v>-0.008924192964144765</v>
+        <v>-0.008924192964144761</v>
       </c>
       <c r="L15" t="n">
-        <v>0.01590378690918018</v>
+        <v>0.01590378690918017</v>
       </c>
       <c r="M15" t="n">
         <v>-0.03043192147242368</v>
       </c>
       <c r="N15" t="n">
-        <v>-0.03422786351058908</v>
+        <v>-0.03422786351058907</v>
       </c>
       <c r="O15" t="n">
         <v>1</v>

</xml_diff>